<commit_message>
feat: add dedicated 'Edit Creditors MSME Data' buttons across Balance Sheet, Note 9 header, and statutory toolbars
</commit_message>
<xml_diff>
--- a/Sample_Statutory_Report_Durga_Steel_Sole_Proprietorship.xlsx
+++ b/Sample_Statutory_Report_Durga_Steel_Sole_Proprietorship.xlsx
@@ -4595,7 +4595,7 @@
         <v>9</v>
       </c>
       <c r="C21" s="18">
-        <v>0</v>
+        <v>420000</v>
       </c>
       <c r="D21" s="18">
         <v>0</v>
@@ -4609,7 +4609,7 @@
         <v>9</v>
       </c>
       <c r="C22" s="18">
-        <v>1821090.23</v>
+        <v>1401090.23</v>
       </c>
       <c r="D22" s="18">
         <v>0</v>
@@ -8080,7 +8080,7 @@
         <v>MSME Creditors</v>
       </c>
       <c r="E106" s="78">
-        <v>0</v>
+        <v>420000</v>
       </c>
       <c r="F106" s="78">
         <v>0</v>
@@ -8100,7 +8100,7 @@
         <v>Other Creditors</v>
       </c>
       <c r="E107" s="82">
-        <v>1821090.23</v>
+        <v>1401090.23</v>
       </c>
       <c r="F107" s="82">
         <v>0</v>
@@ -8140,7 +8140,7 @@
         <v>MSMED Section 22</v>
       </c>
       <c r="E109" s="78">
-        <v>0</v>
+        <v>420000</v>
       </c>
       <c r="F109" s="78">
         <v>0</v>
@@ -8274,7 +8274,7 @@
         <v>(i) MSME</v>
       </c>
       <c r="C116" s="78">
-        <v>0</v>
+        <v>420000</v>
       </c>
       <c r="D116" s="78">
         <v>0</v>
@@ -8283,7 +8283,7 @@
         <v>0</v>
       </c>
       <c r="F116" s="94">
-        <v>0</v>
+        <v>420000</v>
       </c>
     </row>
     <row r="117" ht="20" customHeight="1">
@@ -8294,16 +8294,16 @@
         <v>(ii) Others</v>
       </c>
       <c r="C117" s="82">
-        <v>1821090.23</v>
+        <v>1350000</v>
       </c>
       <c r="D117" s="82">
-        <v>0</v>
+        <v>51090.23</v>
       </c>
       <c r="E117" s="82">
         <v>0</v>
       </c>
       <c r="F117" s="95">
-        <v>1821090.23</v>
+        <v>1401090.23</v>
       </c>
     </row>
     <row r="118" ht="20" customHeight="1">
@@ -8354,10 +8354,10 @@
         <v>Total Trade Payables Aging</v>
       </c>
       <c r="C120" s="21">
-        <v>1821090.23</v>
+        <v>1770000</v>
       </c>
       <c r="D120" s="21">
-        <v>0</v>
+        <v>51090.23</v>
       </c>
       <c r="E120" s="21">
         <v>0</v>

</xml_diff>